<commit_message>
Fix EN/MN data alignment for 3 datasets
- Fix CSV row ordering: sort both EN and MN files consistently by year
  and English category name to ensure numeric values align row-by-row
- Update MN CSV headers to use Mongolian column names for
  inbound-passengers-by-purpose dataset
- Update inbound-passengers-by-purpose-mn.json chart to use Mongolian
  field names (он, зорилго, зорчигч)
- Regenerate XLSX files in wide format (years as columns)

Datasets fixed:
- inbound-passengers-by-purpose
- inbound-passengers-by-region
- university-graduates-by-field

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data.mn/public/datasets/university-graduates-by-field.xlsx
+++ b/data.mn/public/datasets/university-graduates-by-field.xlsx
@@ -1,13 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EN" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MN" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +46,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,287 +426,571 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="35" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="35" customWidth="1" min="8" max="8"/>
-    <col width="35" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="35" customWidth="1" min="11" max="11"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C1" s="1" t="n">
+        <v>2020</v>
+      </c>
+      <c r="D1" s="1" t="n">
+        <v>2021</v>
+      </c>
+      <c r="E1" s="1" t="n">
+        <v>2022</v>
+      </c>
+      <c r="F1" s="1" t="n">
+        <v>2023</v>
+      </c>
+      <c r="G1" s="1" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Agriculture, forestry, fisheries and veterinary</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="B2" t="n">
+        <v>397</v>
+      </c>
+      <c r="C2" t="n">
+        <v>407</v>
+      </c>
+      <c r="D2" t="n">
+        <v>348</v>
+      </c>
+      <c r="E2" t="n">
+        <v>295</v>
+      </c>
+      <c r="F2" t="n">
+        <v>271</v>
+      </c>
+      <c r="G2" t="n">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Arts and humanities</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="B3" t="n">
+        <v>1741</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2127</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2317</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1545</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1759</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1934</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Business, administration and law</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="B4" t="n">
+        <v>9462</v>
+      </c>
+      <c r="C4" t="n">
+        <v>9794</v>
+      </c>
+      <c r="D4" t="n">
+        <v>10506</v>
+      </c>
+      <c r="E4" t="n">
+        <v>7194</v>
+      </c>
+      <c r="F4" t="n">
+        <v>8816</v>
+      </c>
+      <c r="G4" t="n">
+        <v>6433</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Education</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="B5" t="n">
+        <v>5513</v>
+      </c>
+      <c r="C5" t="n">
+        <v>6296</v>
+      </c>
+      <c r="D5" t="n">
+        <v>6001</v>
+      </c>
+      <c r="E5" t="n">
+        <v>3535</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4229</v>
+      </c>
+      <c r="G5" t="n">
+        <v>3151</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Engineering, manufacturing and construction</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="B6" t="n">
+        <v>4306</v>
+      </c>
+      <c r="C6" t="n">
+        <v>4061</v>
+      </c>
+      <c r="D6" t="n">
+        <v>4225</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2910</v>
+      </c>
+      <c r="F6" t="n">
+        <v>3118</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2701</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Health and welfare</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="B7" t="n">
+        <v>3276</v>
+      </c>
+      <c r="C7" t="n">
+        <v>3661</v>
+      </c>
+      <c r="D7" t="n">
+        <v>4293</v>
+      </c>
+      <c r="E7" t="n">
+        <v>4455</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4779</v>
+      </c>
+      <c r="G7" t="n">
+        <v>4886</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Information and Communication Technologies</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="B8" t="n">
+        <v>867</v>
+      </c>
+      <c r="C8" t="n">
+        <v>887</v>
+      </c>
+      <c r="D8" t="n">
+        <v>882</v>
+      </c>
+      <c r="E8" t="n">
+        <v>690</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1082</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1230</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Natural sciences, mathematics and statistics</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="B9" t="n">
+        <v>745</v>
+      </c>
+      <c r="C9" t="n">
+        <v>864</v>
+      </c>
+      <c r="D9" t="n">
+        <v>767</v>
+      </c>
+      <c r="E9" t="n">
+        <v>476</v>
+      </c>
+      <c r="F9" t="n">
+        <v>522</v>
+      </c>
+      <c r="G9" t="n">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Services</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="B10" t="n">
+        <v>455</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1260</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1685</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1277</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1330</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Social sciences, journalism and information</t>
         </is>
       </c>
+      <c r="B11" t="n">
+        <v>1283</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1804</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1901</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1194</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1702</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1424</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>чиглэл</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C1" s="1" t="n">
+        <v>2020</v>
+      </c>
+      <c r="D1" s="1" t="n">
+        <v>2021</v>
+      </c>
+      <c r="E1" s="1" t="n">
+        <v>2022</v>
+      </c>
+      <c r="F1" s="1" t="n">
+        <v>2023</v>
+      </c>
+      <c r="G1" s="1" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>2024</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Байгалийн шинжлэх ухаан, математик, статистик</t>
+        </is>
       </c>
       <c r="B2" t="n">
-        <v>255</v>
+        <v>745</v>
       </c>
       <c r="C2" t="n">
-        <v>1934</v>
+        <v>864</v>
       </c>
       <c r="D2" t="n">
+        <v>767</v>
+      </c>
+      <c r="E2" t="n">
+        <v>476</v>
+      </c>
+      <c r="F2" t="n">
+        <v>522</v>
+      </c>
+      <c r="G2" t="n">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Бизнес, удирдахуй, хууль, эрх зүй</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>9462</v>
+      </c>
+      <c r="C3" t="n">
+        <v>9794</v>
+      </c>
+      <c r="D3" t="n">
+        <v>10506</v>
+      </c>
+      <c r="E3" t="n">
+        <v>7194</v>
+      </c>
+      <c r="F3" t="n">
+        <v>8816</v>
+      </c>
+      <c r="G3" t="n">
         <v>6433</v>
       </c>
-      <c r="E2" t="n">
-        <v>3151</v>
-      </c>
-      <c r="F2" t="n">
-        <v>2701</v>
-      </c>
-      <c r="G2" t="n">
-        <v>4886</v>
-      </c>
-      <c r="H2" t="n">
-        <v>1230</v>
-      </c>
-      <c r="I2" t="n">
-        <v>424</v>
-      </c>
-      <c r="J2" t="n">
-        <v>1330</v>
-      </c>
-      <c r="K2" t="n">
-        <v>1424</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2023</v>
-      </c>
-      <c r="B3" t="n">
-        <v>271</v>
-      </c>
-      <c r="C3" t="n">
-        <v>1759</v>
-      </c>
-      <c r="D3" t="n">
-        <v>8816</v>
-      </c>
-      <c r="E3" t="n">
-        <v>4229</v>
-      </c>
-      <c r="F3" t="n">
-        <v>3118</v>
-      </c>
-      <c r="G3" t="n">
-        <v>4779</v>
-      </c>
-      <c r="H3" t="n">
-        <v>1082</v>
-      </c>
-      <c r="I3" t="n">
-        <v>522</v>
-      </c>
-      <c r="J3" t="n">
-        <v>1277</v>
-      </c>
-      <c r="K3" t="n">
-        <v>1702</v>
-      </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>2022</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Боловсрол</t>
+        </is>
       </c>
       <c r="B4" t="n">
-        <v>295</v>
+        <v>5513</v>
       </c>
       <c r="C4" t="n">
-        <v>1545</v>
+        <v>6296</v>
       </c>
       <c r="D4" t="n">
-        <v>7194</v>
+        <v>6001</v>
       </c>
       <c r="E4" t="n">
         <v>3535</v>
       </c>
       <c r="F4" t="n">
+        <v>4229</v>
+      </c>
+      <c r="G4" t="n">
+        <v>3151</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Инженер, үйлдвэрлэл, барилга угсралт</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4306</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4061</v>
+      </c>
+      <c r="D5" t="n">
+        <v>4225</v>
+      </c>
+      <c r="E5" t="n">
         <v>2910</v>
       </c>
-      <c r="G4" t="n">
+      <c r="F5" t="n">
+        <v>3118</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2701</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Мэдээлэл, харилцаа холбооны технологи</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>867</v>
+      </c>
+      <c r="C6" t="n">
+        <v>887</v>
+      </c>
+      <c r="D6" t="n">
+        <v>882</v>
+      </c>
+      <c r="E6" t="n">
+        <v>690</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1082</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1230</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Нийгмийн шинжлэх ухаан, мэдээлэл, сэтгүүл зүй</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1283</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1804</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1901</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1194</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1702</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1424</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Урлаг, хүмүүнлэг</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1741</v>
+      </c>
+      <c r="C8" t="n">
+        <v>2127</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2317</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1545</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1759</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1934</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Хөдөө аж ахуй, ой, загасны аж ахуй, мал эмнэлэг</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>397</v>
+      </c>
+      <c r="C9" t="n">
+        <v>407</v>
+      </c>
+      <c r="D9" t="n">
+        <v>348</v>
+      </c>
+      <c r="E9" t="n">
+        <v>295</v>
+      </c>
+      <c r="F9" t="n">
+        <v>271</v>
+      </c>
+      <c r="G9" t="n">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Эрүүл мэнд, нийгмийн хамгаалал</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>3276</v>
+      </c>
+      <c r="C10" t="n">
+        <v>3661</v>
+      </c>
+      <c r="D10" t="n">
+        <v>4293</v>
+      </c>
+      <c r="E10" t="n">
         <v>4455</v>
       </c>
-      <c r="H4" t="n">
-        <v>690</v>
-      </c>
-      <c r="I4" t="n">
-        <v>476</v>
-      </c>
-      <c r="J4" t="n">
+      <c r="F10" t="n">
+        <v>4779</v>
+      </c>
+      <c r="G10" t="n">
+        <v>4886</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Үйлчилгээ</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>455</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1260</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1685</v>
+      </c>
+      <c r="E11" t="n">
         <v>1020</v>
       </c>
-      <c r="K4" t="n">
-        <v>1194</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B5" t="n">
-        <v>348</v>
-      </c>
-      <c r="C5" t="n">
-        <v>2317</v>
-      </c>
-      <c r="D5" t="n">
-        <v>10506</v>
-      </c>
-      <c r="E5" t="n">
-        <v>6001</v>
-      </c>
-      <c r="F5" t="n">
-        <v>4225</v>
-      </c>
-      <c r="G5" t="n">
-        <v>4293</v>
-      </c>
-      <c r="H5" t="n">
-        <v>882</v>
-      </c>
-      <c r="I5" t="n">
-        <v>767</v>
-      </c>
-      <c r="J5" t="n">
-        <v>1685</v>
-      </c>
-      <c r="K5" t="n">
-        <v>1901</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>2020</v>
-      </c>
-      <c r="B6" t="n">
-        <v>407</v>
-      </c>
-      <c r="C6" t="n">
-        <v>2127</v>
-      </c>
-      <c r="D6" t="n">
-        <v>9794</v>
-      </c>
-      <c r="E6" t="n">
-        <v>6296</v>
-      </c>
-      <c r="F6" t="n">
-        <v>4061</v>
-      </c>
-      <c r="G6" t="n">
-        <v>3661</v>
-      </c>
-      <c r="H6" t="n">
-        <v>887</v>
-      </c>
-      <c r="I6" t="n">
-        <v>864</v>
-      </c>
-      <c r="J6" t="n">
-        <v>1260</v>
-      </c>
-      <c r="K6" t="n">
-        <v>1804</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>2019</v>
-      </c>
-      <c r="B7" t="n">
-        <v>397</v>
-      </c>
-      <c r="C7" t="n">
-        <v>1741</v>
-      </c>
-      <c r="D7" t="n">
-        <v>9462</v>
-      </c>
-      <c r="E7" t="n">
-        <v>5513</v>
-      </c>
-      <c r="F7" t="n">
-        <v>4306</v>
-      </c>
-      <c r="G7" t="n">
-        <v>3276</v>
-      </c>
-      <c r="H7" t="n">
-        <v>867</v>
-      </c>
-      <c r="I7" t="n">
-        <v>745</v>
-      </c>
-      <c r="J7" t="n">
-        <v>455</v>
-      </c>
-      <c r="K7" t="n">
-        <v>1283</v>
+      <c r="F11" t="n">
+        <v>1277</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1330</v>
       </c>
     </row>
   </sheetData>

</xml_diff>